<commit_message>
Scrapper is now headless
</commit_message>
<xml_diff>
--- a/Scraper/PSU_Student_Organizations.xlsx
+++ b/Scraper/PSU_Student_Organizations.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/msalau/Desktop/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5A58A080-F022-1D43-9472-797ACD0685B3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E0AB9C78-1965-D94C-BCCF-4CFD63B2A7C0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="500" windowWidth="28800" windowHeight="16340" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="500" windowWidth="28800" windowHeight="15800" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Student Organizations" sheetId="1" r:id="rId1"/>

</xml_diff>